<commit_message>
Update data package at: 2026-09-21T07:23:18Z
</commit_message>
<xml_diff>
--- a/data-raw/Nome_UO_antigas.xlsx
+++ b/data-raw/Nome_UO_antigas.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>cod_uo</t>
   </si>
@@ -43,19 +43,7 @@
     <t>nome</t>
   </si>
   <si>
-    <t>ESCRITÓRIO DE REPRESENTAÇÃO DO GOVERNO DO ESTADO DE MINAS GERAIS NO RIO DE JANEIRO - ERRJ</t>
-  </si>
-  <si>
-    <t>ESCRITÓRIO DE REPRESENTAÇÃO DO GOVERNO DO ESTADO DE MINAS GERAIS EM SÃO PAULO - ERSP</t>
-  </si>
-  <si>
-    <t>ESCRITÓRIO DE PRIORIDADES ESTRATÉGICAS - EPE</t>
-  </si>
-  <si>
     <t>SECRETARIA DE ESTADO DE SAÚDE - SES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEPARTAMENTO DE TRÂNSITO DE MINAS GERAIS - DETRAN </t>
   </si>
 </sst>
 </file>
@@ -397,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="91" customWidth="1"/>
@@ -413,42 +401,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1141</v>
+        <v>1320</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1161</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1601</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>1320</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>1551</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -458,14 +414,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -730,27 +684,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F4F70FD-B48D-426A-882C-1E2AF784F4D5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26681440-2F92-4A6D-B6E4-616C75823A42}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -775,9 +722,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26681440-2F92-4A6D-B6E4-616C75823A42}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F4F70FD-B48D-426A-882C-1E2AF784F4D5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>